<commit_message>
Catálogo: Tiara en Cadenas y collares y cruces con o sin cadena
El plazo a pedido es de 15 a 20 días corridos; en la web se dice
"entre 15 y 20 días".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/productos.xlsx
+++ b/catalogo/productos.xlsx
@@ -656,7 +656,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Las 10 filas de la hoja Productos son los 8 productos reales de partida (dos de ellos con versiones). Faltan precio, tamaño y descripción.</t>
+          <t>Las 12 filas de la hoja Productos son los 8 productos reales de partida (las cruces y las medallas, con y sin cadena). Faltan precio, tamaño y descripción.</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -776,7 +776,11 @@
           <t>Bronce</t>
         </is>
       </c>
-      <c r="F2" s="7" t="n"/>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Con cadena</t>
+        </is>
+      </c>
       <c r="G2" s="8" t="n"/>
       <c r="H2" s="9" t="n"/>
       <c r="I2" s="7" t="n"/>
@@ -791,50 +795,34 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>cruz-victoria-plata-lisa</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Cruz de la Victoria en plata lisa</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Colección Astur</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Colgantes</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Plata</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="n"/>
+          <t>cruz-victoria-bronce-circones</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n"/>
+      <c r="C3" s="11" t="n"/>
+      <c r="D3" s="11" t="n"/>
+      <c r="E3" s="11" t="n"/>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Sin cadena</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="n"/>
-      <c r="H3" s="9" t="n"/>
-      <c r="I3" s="7" t="n"/>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>Borrador</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="n"/>
+      <c r="H3" s="11" t="n"/>
+      <c r="I3" s="11" t="n"/>
+      <c r="J3" s="12" t="n"/>
+      <c r="K3" s="11" t="n"/>
+      <c r="L3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>medalla-covadonga-bronce</t>
+          <t>cruz-victoria-plata-lisa</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Medalla Virgen de Covadonga en bronce</t>
+          <t>Cruz de la Victoria en plata lisa</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -849,7 +837,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Bronce</t>
+          <t>Plata</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -866,16 +854,12 @@
           <t>Borrador</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>Versiones con y sin cadena: confirmar.</t>
-        </is>
-      </c>
+      <c r="L4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>medalla-covadonga-bronce</t>
+          <t>cruz-victoria-plata-lisa</t>
         </is>
       </c>
       <c r="B5" s="11" t="n"/>
@@ -897,12 +881,12 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>medalla-covadonga-plata</t>
+          <t>medalla-covadonga-bronce</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Medalla Virgen de Covadonga en plata</t>
+          <t>Medalla Virgen de Covadonga en bronce</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -917,7 +901,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Plata</t>
+          <t>Bronce</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -934,16 +918,12 @@
           <t>Borrador</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>Versiones con y sin cadena: confirmar.</t>
-        </is>
-      </c>
+      <c r="L6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>medalla-covadonga-plata</t>
+          <t>medalla-covadonga-bronce</t>
         </is>
       </c>
       <c r="B7" s="11" t="n"/>
@@ -965,30 +945,34 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>cadena-clasica-bronce</t>
+          <t>medalla-covadonga-plata</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Cadena clásica en bronce</t>
+          <t>Medalla Virgen de Covadonga en plata</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Sin colección</t>
+          <t>Colección Astur</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Cadenas y collares</t>
+          <t>Colgantes</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Bronce</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="n"/>
+          <t>Plata</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Con cadena</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="7" t="n"/>
@@ -1003,50 +987,34 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>cadena-clasica-plata</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Cadena clásica en plata</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Sin colección</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Cadenas y collares</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Plata</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="n"/>
+          <t>medalla-covadonga-plata</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Sin cadena</t>
+        </is>
+      </c>
       <c r="G9" s="8" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="10" t="n"/>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>Borrador</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="11" t="n"/>
+      <c r="J9" s="12" t="n"/>
+      <c r="K9" s="11" t="n"/>
+      <c r="L9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>tiara-bronce</t>
+          <t>cadena-clasica-bronce</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Tiara en bronce</t>
+          <t>Cadena clásica en bronce</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -1054,7 +1022,11 @@
           <t>Sin colección</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Cadenas y collares</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Bronce</t>
@@ -1070,21 +1042,17 @@
           <t>Borrador</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr">
-        <is>
-          <t>Falta definir su categoría.</t>
-        </is>
-      </c>
+      <c r="L10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>colgante-bronce-onix</t>
+          <t>cadena-clasica-plata</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Colgante de bronce con piedra ónix</t>
+          <t>Cadena clásica en plata</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1094,12 +1062,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Colgantes</t>
+          <t>Cadenas y collares</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Bronce</t>
+          <t>Plata</t>
         </is>
       </c>
       <c r="F11" s="7" t="n"/>
@@ -1113,6 +1081,82 @@
         </is>
       </c>
       <c r="L11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>tiara-bronce</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tiara en bronce</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Sin colección</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Cadenas y collares</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Bronce</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="7" t="n"/>
+      <c r="J12" s="10" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>colgante-bronce-onix</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Colgante de bronce con piedra ónix</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Sin colección</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Colgantes</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Bronce</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="7" t="n"/>
+      <c r="J13" s="10" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="5">

</xml_diff>

<commit_message>
Catálogo: categorías Anillos, Aros, Esclavas y Pulseras
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/productos.xlsx
+++ b/catalogo/productos.xlsx
@@ -646,7 +646,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>• Colecciones vigentes: Colección Astur. Categorías vigentes: Cadenas y collares, Colgantes.</t>
+          <t>• Colecciones vigentes: Colección Astur. Categorías vigentes: Anillos, Aros, Cadenas y collares, Colgantes, Esclavas y Pulseras.</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Cadenas y collares</t>
+          <t>Anillos</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
@@ -1248,17 +1248,45 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
+          <t>Aros</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Plata</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Publicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cadenas y collares</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Colgantes</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
-        <is>
-          <t>Plata</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr">
-        <is>
-          <t>Publicado</t>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Esclavas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pulseras</t>
         </is>
       </c>
     </row>

</xml_diff>